<commit_message>
Extend pivot fill draft to all 84 built-in presets
Change-Id: I11ef3a574d187549f4ca9ae521fafd52ced20371
</commit_message>
<xml_diff>
--- a/esilk/repro/pivot-banding/both-axes-control.xlsx
+++ b/esilk/repro/pivot-banding/both-axes-control.xlsx
@@ -157,74 +157,74 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HandmadePivot" cacheId="1" dataCaption="Values" rowGrandTotals="1" colGrandTotals="1" compact="0" compactData="0" outline="0" outlineData="0" gridDropZones="1">
-  <location ref="B3:G8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="3">
-    <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x v="0"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x v="0"/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="5">
-    <i>
-      <x v="0"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x v="0"/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Value" fld="2" subtotal="sum"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="1" showColStripes="1"/>
-</pivotTableDefinition>
+<ns0:pivotTableDefinition xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="HandmadePivot" cacheId="1" dataCaption="Values" rowGrandTotals="1" colGrandTotals="1" compact="0" compactData="0" outline="0" outlineData="0" gridDropZones="1">
+  <ns0:location ref="B3:G8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <ns0:pivotFields count="3">
+    <ns0:pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
+      <ns0:items count="5">
+        <ns0:item x="0"/>
+        <ns0:item x="1"/>
+        <ns0:item x="2"/>
+        <ns0:item x="3"/>
+        <ns0:item t="default"/>
+      </ns0:items>
+    </ns0:pivotField>
+    <ns0:pivotField axis="axisCol" showAll="0" defaultSubtotal="0">
+      <ns0:items count="5">
+        <ns0:item x="0"/>
+        <ns0:item x="1"/>
+        <ns0:item x="2"/>
+        <ns0:item x="3"/>
+        <ns0:item t="default"/>
+      </ns0:items>
+    </ns0:pivotField>
+    <ns0:pivotField dataField="1" showAll="0"/>
+  </ns0:pivotFields>
+  <ns0:rowFields count="1">
+    <ns0:field x="0"/>
+  </ns0:rowFields>
+  <ns0:rowItems count="5">
+    <ns0:i>
+      <ns0:x v="0"/>
+    </ns0:i>
+    <ns0:i>
+      <ns0:x v="1"/>
+    </ns0:i>
+    <ns0:i>
+      <ns0:x v="2"/>
+    </ns0:i>
+    <ns0:i>
+      <ns0:x v="3"/>
+    </ns0:i>
+    <ns0:i t="grand">
+      <ns0:x v="0"/>
+    </ns0:i>
+  </ns0:rowItems>
+  <ns0:colFields count="1">
+    <ns0:field x="1"/>
+  </ns0:colFields>
+  <ns0:colItems count="5">
+    <ns0:i>
+      <ns0:x v="0"/>
+    </ns0:i>
+    <ns0:i>
+      <ns0:x v="1"/>
+    </ns0:i>
+    <ns0:i>
+      <ns0:x v="2"/>
+    </ns0:i>
+    <ns0:i>
+      <ns0:x v="3"/>
+    </ns0:i>
+    <ns0:i t="grand">
+      <ns0:x v="0"/>
+    </ns0:i>
+  </ns0:colItems>
+  <ns0:dataFields count="1">
+    <ns0:dataField name="Sum of Value" fld="2" subtotal="sum"/>
+  </ns0:dataFields>
+  <ns0:pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="1" showColStripes="1" showLastColumn="1"/>
+</ns0:pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>